<commit_message>
Update CrossUse analysis to match real data schema
- Single Excel input (no separate product master)
- Separate column: 自社IP / 他社IP / shoppingbag
- Auto-exclude shoppingbag rows before classification
- Updated sample data to match real column structure

https://claude.ai/code/session_01Xim644LNhEMHWr2TqyN3Bv
</commit_message>
<xml_diff>
--- a/results/crossuse_analysis.xlsx
+++ b/results/crossuse_analysis.xlsx
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,15 +34,13 @@
       <sz val="13"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <sz val="10"/>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
@@ -78,7 +76,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
+        <fgColor rgb="00F5F5F5"/>
       </patternFill>
     </fill>
     <fill>
@@ -128,15 +126,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -145,37 +146,37 @@
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" indent="1"/>
     </xf>
   </cellXfs>
@@ -543,93 +544,101 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CrossUse分析 ― コラボ×自社IP セグメント集計</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
+          <t>CrossUse分析 ― 他社IP × 自社IP セグメント集計（カート単位）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>※ shoppingbag は集計除外済み　／　1カート（order_id）を1取引として集計</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
           <t>セグメント名</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>注文数</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>注文数（カート）</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>構成比(%)</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>コラボのみ</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="C3" s="5" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>コラボ + 自社IP（同時購入）</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C4" s="5" t="n">
-        <v>0.1</v>
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>他社IP（コラボ）のみ</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>0.4</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>自社IPのみ</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="C5" s="5" t="n">
-        <v>0.4</v>
+          <t>他社IP + 自社IP（クロス購買）</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>0.2</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
+          <t>自社IPのみ</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="B6" s="9" t="n">
+      <c r="B7" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="C6" s="10" t="n">
+      <c r="C7" s="11" t="n">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -645,243 +654,263 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
-        <is>
-          <t>注文ID別 セグメント分類一覧</t>
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>注文ID別 セグメント分類一覧（shoppingbag除外済み）</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>order_id</t>
         </is>
       </c>
-      <c r="B2" s="12" t="inlineStr">
-        <is>
-          <t>コラボ含む</t>
-        </is>
-      </c>
-      <c r="C2" s="12" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>他社IP含む</t>
+        </is>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
         <is>
           <t>自社IP含む</t>
         </is>
       </c>
-      <c r="D2" s="12" t="inlineStr">
+      <c r="D2" s="13" t="inlineStr">
         <is>
           <t>セグメント</t>
         </is>
       </c>
     </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="13" t="n">
-        <v>1001</v>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="C3" s="13" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="D3" s="14" t="inlineStr">
-        <is>
-          <t>コラボ + 自社IP（同時購入）</t>
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>ORD-001</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="inlineStr">
+        <is>
+          <t>―</t>
+        </is>
+      </c>
+      <c r="D3" s="15" t="inlineStr">
+        <is>
+          <t>他社IP（コラボ）のみ</t>
         </is>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="13" t="n">
-        <v>1002</v>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="C4" s="13" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>ORD-002</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>―</t>
         </is>
       </c>
-      <c r="D4" s="15" t="inlineStr">
-        <is>
-          <t>コラボのみ</t>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="D4" s="16" t="inlineStr">
+        <is>
+          <t>自社IPのみ</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="13" t="n">
-        <v>1003</v>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>ORD-003</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="inlineStr">
+        <is>
+          <t>他社IP + 自社IP（クロス購買）</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>ORD-004</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>―</t>
         </is>
       </c>
-      <c r="C5" s="13" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="D5" s="16" t="inlineStr">
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>他社IP（コラボ）のみ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>ORD-005</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>―</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
         <is>
           <t>自社IPのみ</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="13" t="n">
-        <v>1004</v>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="C6" s="13" t="inlineStr">
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>ORD-006</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>―</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
-        <is>
-          <t>コラボのみ</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="13" t="n">
-        <v>1005</v>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>自社IPのみ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>ORD-007</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>他社IP + 自社IP（クロス購買）</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>ORD-008</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>―</t>
         </is>
       </c>
-      <c r="D7" s="15" t="inlineStr">
-        <is>
-          <t>コラボのみ</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="13" t="n">
-        <v>1006</v>
-      </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>他社IP（コラボ）のみ</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>ORD-009</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
         <is>
           <t>―</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="D8" s="16" t="inlineStr">
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
         <is>
           <t>自社IPのみ</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="13" t="n">
-        <v>1007</v>
-      </c>
-      <c r="B9" s="13" t="inlineStr">
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>ORD-010</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>―</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="D9" s="16" t="inlineStr">
-        <is>
-          <t>自社IPのみ</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="13" t="n">
-        <v>1008</v>
-      </c>
-      <c r="B10" s="13" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="C10" s="13" t="inlineStr">
-        <is>
-          <t>―</t>
-        </is>
-      </c>
-      <c r="D10" s="15" t="inlineStr">
-        <is>
-          <t>コラボのみ</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="13" t="n">
-        <v>1009</v>
-      </c>
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>―</t>
-        </is>
-      </c>
-      <c r="C11" s="13" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="D11" s="16" t="inlineStr">
-        <is>
-          <t>自社IPのみ</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="13" t="n">
-        <v>1010</v>
-      </c>
-      <c r="B12" s="13" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="C12" s="13" t="inlineStr">
-        <is>
-          <t>―</t>
-        </is>
-      </c>
       <c r="D12" s="15" t="inlineStr">
         <is>
-          <t>コラボのみ</t>
+          <t>他社IP（コラボ）のみ</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add sales amount columns to CrossUse segment analysis
- Summarize total sales and sales % per segment
- Add sales column to order detail sheet

https://claude.ai/code/session_01Xim644LNhEMHWr2TqyN3Bv
</commit_message>
<xml_diff>
--- a/results/crossuse_analysis.xlsx
+++ b/results/crossuse_analysis.xlsx
@@ -126,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -169,6 +169,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" indent="1"/>
@@ -544,12 +547,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -579,7 +584,17 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>構成比(%)</t>
+          <t>注文構成比</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>売上合計</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>売上構成比</t>
         </is>
       </c>
     </row>
@@ -595,6 +610,12 @@
       <c r="C4" s="6" t="n">
         <v>0.4</v>
       </c>
+      <c r="D4" s="5" t="n">
+        <v>13500</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>0.287</v>
+      </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
@@ -608,6 +629,12 @@
       <c r="C5" s="6" t="n">
         <v>0.2</v>
       </c>
+      <c r="D5" s="5" t="n">
+        <v>12000</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>0.255</v>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -621,6 +648,12 @@
       <c r="C6" s="6" t="n">
         <v>0.4</v>
       </c>
+      <c r="D6" s="5" t="n">
+        <v>21500</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>0.457</v>
+      </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
@@ -634,11 +667,19 @@
       <c r="C7" s="11" t="n">
         <v>1</v>
       </c>
+      <c r="D7" s="10" t="n">
+        <v>47000</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
     <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A2:E2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -650,13 +691,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -684,6 +726,11 @@
       </c>
       <c r="D2" s="13" t="inlineStr">
         <is>
+          <t>売上合計</t>
+        </is>
+      </c>
+      <c r="E2" s="13" t="inlineStr">
+        <is>
           <t>セグメント</t>
         </is>
       </c>
@@ -704,7 +751,10 @@
           <t>―</t>
         </is>
       </c>
-      <c r="D3" s="15" t="inlineStr">
+      <c r="D3" s="15" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E3" s="16" t="inlineStr">
         <is>
           <t>他社IP（コラボ）のみ</t>
         </is>
@@ -726,7 +776,10 @@
           <t>○</t>
         </is>
       </c>
-      <c r="D4" s="16" t="inlineStr">
+      <c r="D4" s="15" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
         <is>
           <t>自社IPのみ</t>
         </is>
@@ -748,7 +801,10 @@
           <t>○</t>
         </is>
       </c>
-      <c r="D5" s="17" t="inlineStr">
+      <c r="D5" s="15" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E5" s="18" t="inlineStr">
         <is>
           <t>他社IP + 自社IP（クロス購買）</t>
         </is>
@@ -770,7 +826,10 @@
           <t>―</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="D6" s="15" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E6" s="16" t="inlineStr">
         <is>
           <t>他社IP（コラボ）のみ</t>
         </is>
@@ -792,7 +851,10 @@
           <t>○</t>
         </is>
       </c>
-      <c r="D7" s="16" t="inlineStr">
+      <c r="D7" s="15" t="n">
+        <v>3500</v>
+      </c>
+      <c r="E7" s="17" t="inlineStr">
         <is>
           <t>自社IPのみ</t>
         </is>
@@ -814,7 +876,10 @@
           <t>○</t>
         </is>
       </c>
-      <c r="D8" s="16" t="inlineStr">
+      <c r="D8" s="15" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
         <is>
           <t>自社IPのみ</t>
         </is>
@@ -836,7 +901,10 @@
           <t>○</t>
         </is>
       </c>
-      <c r="D9" s="17" t="inlineStr">
+      <c r="D9" s="15" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E9" s="18" t="inlineStr">
         <is>
           <t>他社IP + 自社IP（クロス購買）</t>
         </is>
@@ -858,7 +926,10 @@
           <t>―</t>
         </is>
       </c>
-      <c r="D10" s="15" t="inlineStr">
+      <c r="D10" s="15" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E10" s="16" t="inlineStr">
         <is>
           <t>他社IP（コラボ）のみ</t>
         </is>
@@ -880,7 +951,10 @@
           <t>○</t>
         </is>
       </c>
-      <c r="D11" s="16" t="inlineStr">
+      <c r="D11" s="15" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
         <is>
           <t>自社IPのみ</t>
         </is>
@@ -902,7 +976,10 @@
           <t>―</t>
         </is>
       </c>
-      <c r="D12" s="15" t="inlineStr">
+      <c r="D12" s="15" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E12" s="16" t="inlineStr">
         <is>
           <t>他社IP（コラボ）のみ</t>
         </is>

</xml_diff>

<commit_message>
Fix sales calculation: use sales * quantity for line total
Sales column was unit price, not total. Multiply by quantity to get
correct sales amount per line item.

https://claude.ai/code/session_01Xim644LNhEMHWr2TqyN3Bv
</commit_message>
<xml_diff>
--- a/results/crossuse_analysis.xlsx
+++ b/results/crossuse_analysis.xlsx
@@ -611,10 +611,10 @@
         <v>0.4</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>13500</v>
+        <v>19500</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.287</v>
+        <v>0.253</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -633,7 +633,7 @@
         <v>12000</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.255</v>
+        <v>0.156</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -649,10 +649,10 @@
         <v>0.4</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>21500</v>
+        <v>45500</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.457</v>
+        <v>0.591</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>47000</v>
+        <v>77000</v>
       </c>
       <c r="E7" s="11" t="n">
         <v>1</v>
@@ -777,7 +777,7 @@
         </is>
       </c>
       <c r="D4" s="15" t="n">
-        <v>6000</v>
+        <v>12000</v>
       </c>
       <c r="E4" s="17" t="inlineStr">
         <is>
@@ -877,7 +877,7 @@
         </is>
       </c>
       <c r="D8" s="15" t="n">
-        <v>9000</v>
+        <v>27000</v>
       </c>
       <c r="E8" s="17" t="inlineStr">
         <is>
@@ -927,7 +927,7 @@
         </is>
       </c>
       <c r="D10" s="15" t="n">
-        <v>6000</v>
+        <v>12000</v>
       </c>
       <c r="E10" s="16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Simplify sales calc: sales column already contains total amount
Remove quantity multiplication since sales is now pre-calculated
as unit price × quantity.

https://claude.ai/code/session_01Xim644LNhEMHWr2TqyN3Bv
</commit_message>
<xml_diff>
--- a/results/crossuse_analysis.xlsx
+++ b/results/crossuse_analysis.xlsx
@@ -611,10 +611,10 @@
         <v>0.4</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>19500</v>
+        <v>13500</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.253</v>
+        <v>0.287</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -633,7 +633,7 @@
         <v>12000</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.156</v>
+        <v>0.255</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -649,10 +649,10 @@
         <v>0.4</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>45500</v>
+        <v>21500</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.591</v>
+        <v>0.457</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -668,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>77000</v>
+        <v>47000</v>
       </c>
       <c r="E7" s="11" t="n">
         <v>1</v>
@@ -777,7 +777,7 @@
         </is>
       </c>
       <c r="D4" s="15" t="n">
-        <v>12000</v>
+        <v>6000</v>
       </c>
       <c r="E4" s="17" t="inlineStr">
         <is>
@@ -877,7 +877,7 @@
         </is>
       </c>
       <c r="D8" s="15" t="n">
-        <v>27000</v>
+        <v>9000</v>
       </c>
       <c r="E8" s="17" t="inlineStr">
         <is>
@@ -927,7 +927,7 @@
         </is>
       </c>
       <c r="D10" s="15" t="n">
-        <v>12000</v>
+        <v>6000</v>
       </c>
       <c r="E10" s="16" t="inlineStr">
         <is>

</xml_diff>